<commit_message>
Added defects to defect report with reference links
</commit_message>
<xml_diff>
--- a/FM_G10_Defect report_template.xlsx
+++ b/FM_G10_Defect report_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\Desktop\FM_Seminarski_rad_G10\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\senad\FM_Seminarski_rad_G10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB5762D-4D69-4EF9-B7B9-468F107D96EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9805CF81-C172-413C-A109-28B70A099CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Defect Tracking Log" sheetId="1" r:id="rId1"/>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="84">
   <si>
     <r>
       <rPr>
@@ -410,10 +410,46 @@
     <t>Funkcionalnost pretrage i filtriranja ne vrši validaciju raspona cijene kada je minimalna cijena veća od maksimalne. Sistem prikazuje poruku "Nema rezultata", umjesto da upozori korisnika na neispravan unos, što može dovesti do konfuzije. Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/benjamin_muratovic_edu_fit_ba/IQDAELXUqnNaSoaWvqyFO-NaAdo4xLmpLhtCdddijx4RNr4?e=bqj0x5</t>
   </si>
   <si>
-    <t>Funkcionalnost pretrage dozvoljava unos specijalnih karaktera (npr. %&amp;%) bez ikakve validacije. Sistem prikazuje poruku "Nema rezultata" umjesto da obavijesti korisnika da je unos neispravan, što ovodi do nejasnog ponašanja sistema. Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/benjamin_muratovic_edu_fit_ba/IQCpLaDK-IWxRYFMy8sVSp7bAW-VazjE8EvErw3_4ITW88Q?e=7vPaax</t>
-  </si>
-  <si>
-    <t>Funkcionalnost pretrage ne nudi prijedlog ili alternativne rezultate kada korisnik napravi manju tipografsku grešku u pojmu za pretragu (npr. „iphne“ umjesto „iphone“), već odmah prikazuje poruku „Nema rezultata“, što negativno utiče na korisničko iskustvo. Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/benjamin_muratovic_edu_fit_ba/IQCvonx9eof6Q4yXn84lDV-hAZ5-R_48YEnO8L3qhoVjquY?e=FAaYvB</t>
+    <t>06.01.2026.</t>
+  </si>
+  <si>
+    <t>Selma Alagić</t>
+  </si>
+  <si>
+    <t>Ograničiti ili validirati unos cijene i prikazati korisniku jasnu poruku ako unesena vrijednost nije ispravna, a ako je raspon cijene validan, prikazati relevantne rezultate za taj filter.</t>
+  </si>
+  <si>
+    <t>Funkcionalnost pretrage ne nudi prijedlog ili alternativne rezultate kada korisnik napravi manju tipografsku grešku u pojmu za pretragu (npr. „iphne“ umjesto „iphone“), već odmah prikazuje poruku „Nema rezultata“, što negativno utiče na korisničko iskustvo.
+Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/benjamin_muratovic_edu_fit_ba/IQCvonx9eof6Q4yXn84lDV-hAZ5-R_48YEnO8L3qhoVjquY?e=FAaYvB</t>
+  </si>
+  <si>
+    <t>Funkcionalnost pretrage dozvoljava unos specijalnih karaktera (npr. %&amp;%) bez ikakve validacije. Sistem prikazuje poruku "Nema rezultata" umjesto da obavijesti korisnika da je unos neispravan, što ovodi do nejasnog ponašanja sistema.
+Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/benjamin_muratovic_edu_fit_ba/IQCpLaDK-IWxRYFMy8sVSp7bAW-VazjE8EvErw3_4ITW88Q?e=7vPaax</t>
+  </si>
+  <si>
+    <t>Funkcionalnost filtriranja proizvoda prema unesenoj cijeni (od/do) se ne izvršava ispravno u slučaju kada unesemo da je cijena od:0 i do:0. Ukoliko odaberemo bilo koju kategoriju i filtriramo proizvode prema cijeni na taj način, sistem ni na koji način ne obavještava korisnike da proizvod u tom opsegu cijene i odabranoj kategoriji ne postoji već prikaže proizvode odabrane kategorije sa nasumičnim cijenama koje ne odgovaraju zadanom filteru. 
+Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/alagic_selma_edu_fit_ba/IQA99-mhH8N3QIWCzYJ7a_TXASjWGLenJ4i4WkfZAaxz6Rc?nav=eyJyZWZlcnJhbEluZm8iOnsicmVmZXJyYWxBcHAiOiJPbmVEcml2ZUZvckJ1c2luZXNzIiwicmVmZXJyYWxBcHBQbGF0Zm9ybSI6IldlYiIsInJlZmVycmFsTW9kZSI6InZpZXciLCJyZWZlcnJhbFZpZXciOiJNeUZpbGVzTGlua0NvcHkifX0&amp;e=nEUFsN</t>
+  </si>
+  <si>
+    <t>Funkcionalnost resetovanja svih filtera (tj. opcija “Clear All”) trenutno nije dostupna. Kada korisnici odaberu više filtera (npr. cijena, lokacija, proizvođač), moraju ih uklanjati jedan po jedan, iako bi možda željeli ukloniti sve odjednom i odabrati nove vrijednosti ili početi novu pretragu. Ovo nije optimalno korisničko iskustvo jer povećava broj klikova, usporava pretragu i može biti frustrirajuće, posebno ako korisnik želi brzo promijeniti kriterije pretrage.
+Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/alagic_selma_edu_fit_ba/IQCoCCvWqQIoTosPBN6pwZS8Af_wX0ANCYYx8qFbx1_Y3fU?nav=eyJyZWZlcnJhbEluZm8iOnsicmVmZXJyYWxBcHAiOiJPbmVEcml2ZUZvckJ1c2luZXNzIiwicmVmZXJyYWxBcHBQbGF0Zm9ybSI6IldlYiIsInJlZmVycmFsTW9kZSI6InZpZXciLCJyZWZlcnJhbFZpZXciOiJNeUZpbGVzTGlua0NvcHkifX0&amp;e=kznKW3</t>
+  </si>
+  <si>
+    <t>Dodati opciju “Clear All”  koja će biti jasno vidljiva korisnicima i omogućiti uklanjanje svih filtera odjednom, čime će se poboljšava efikasnost pretrage i zadovoljstvo korisnika.</t>
+  </si>
+  <si>
+    <t>Polje za unos ključnih riječi kod pretrage proizvoda nema ograničenje unosa karaktera. Maksimalni podržani broj karaktera je 255, ali ako se unese više (npr. 270), sistem korisnicima prikazuje poruku ‘nema rezultata’ bez bilo kakvog upozorenja da je unos izvan dozvoljenog opsega.
+Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/alagic_selma_edu_fit_ba/IQCV2j3WZyJ0TqaAUo2t-ctRAfyvKNIv2n74mKO0H18zF0c?nav=eyJyZWZlcnJhbEluZm8iOnsicmVmZXJyYWxBcHAiOiJPbmVEcml2ZUZvckJ1c2luZXNzIiwicmVmZXJyYWxBcHBQbGF0Zm9ybSI6IldlYiIsInJlZmVycmFsTW9kZSI6InZpZXciLCJyZWZlcnJhbFZpZXciOiJNeUZpbGVzTGlua0NvcHkifX0&amp;e=h5eted</t>
+  </si>
+  <si>
+    <t>Prikazati korisniku upozorenje ili validacijsku poruku ukoliko pokuša unijeti više od dozvoljenog broja karaktera.</t>
+  </si>
+  <si>
+    <t>Kada korisnik pretražuje proizvod koji ne postoji i ne koristi nikakve filtere, opcija ‘Očisti filtere’ se pojavljuje tek kada nema rezultata za pretragu. Ovo može zbuniti korisnika jer nije primijenio nikakve filtere, a opcija za njihovo uklanjanje se bespotrebno prikazuje.
+Link za showcase: https://edufit-my.sharepoint.com/:v:/g/personal/alagic_selma_edu_fit_ba/IQDlqIIQqC6aR66YgHYnmd2NAU6A3tKtVRcIual61Gam2zI?nav=eyJyZWZlcnJhbEluZm8iOnsicmVmZXJyYWxBcHAiOiJPbmVEcml2ZUZvckJ1c2luZXNzIiwicmVmZXJyYWxBcHBQbGF0Zm9ybSI6IldlYiIsInJlZmVycmFsTW9kZSI6InZpZXciLCJyZWZlcnJhbFZpZXciOiJNeUZpbGVzTGlua0NvcHkifX0&amp;e=T7HmaH</t>
+  </si>
+  <si>
+    <t>Opcija ‘Očisti filtere’ treba se prikazivati samo kada su filteri aktivni. Ako korisnik nije primijenio nijedan filter, opcija se ne prikazuje, čak ni kada nema rezultata pretrage.</t>
   </si>
 </sst>
 </file>
@@ -833,7 +869,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
@@ -893,25 +929,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -933,26 +950,57 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1175,7 +1223,7 @@
     <col min="1" max="1" width="20.44140625" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" customWidth="1"/>
     <col min="3" max="3" width="17.109375" customWidth="1"/>
-    <col min="4" max="4" width="41.88671875" customWidth="1"/>
+    <col min="4" max="4" width="44.44140625" customWidth="1"/>
     <col min="5" max="5" width="11.44140625" customWidth="1"/>
     <col min="6" max="6" width="15.44140625" customWidth="1"/>
     <col min="7" max="7" width="7.44140625" customWidth="1"/>
@@ -1195,23 +1243,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
-      <c r="N1" s="30"/>
-      <c r="O1" s="30"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="38"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="38"/>
+      <c r="K1" s="38"/>
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+      <c r="N1" s="38"/>
+      <c r="O1" s="38"/>
     </row>
     <row r="2" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1249,43 +1297,43 @@
     </row>
     <row r="6" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:24" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="31" t="s">
+      <c r="A7" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="32"/>
-      <c r="K7" s="32"/>
-      <c r="L7" s="32"/>
-      <c r="M7" s="32"/>
-      <c r="N7" s="32"/>
-      <c r="O7" s="32"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="40"/>
+      <c r="D7" s="40"/>
+      <c r="E7" s="40"/>
+      <c r="F7" s="40"/>
+      <c r="G7" s="40"/>
+      <c r="H7" s="40"/>
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="40"/>
+      <c r="L7" s="40"/>
+      <c r="M7" s="40"/>
+      <c r="N7" s="40"/>
+      <c r="O7" s="40"/>
       <c r="P7" s="3"/>
     </row>
     <row r="8" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="32"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="32"/>
-      <c r="N8" s="32"/>
-      <c r="O8" s="32"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="40"/>
+      <c r="I8" s="40"/>
+      <c r="J8" s="40"/>
+      <c r="K8" s="40"/>
+      <c r="L8" s="40"/>
+      <c r="M8" s="40"/>
+      <c r="N8" s="40"/>
+      <c r="O8" s="40"/>
     </row>
     <row r="9" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="10" spans="1:24" ht="39.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
@@ -1347,66 +1395,66 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:24" ht="118.8" x14ac:dyDescent="0.25">
-      <c r="A11" s="46">
+    <row r="11" spans="1:24" ht="129.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="49">
         <v>1</v>
       </c>
-      <c r="B11" s="38">
-        <v>46174</v>
-      </c>
-      <c r="C11" s="39" t="s">
+      <c r="B11" s="55" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="50" t="s">
         <v>67</v>
       </c>
-      <c r="D11" s="48" t="s">
+      <c r="D11" s="53" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="39"/>
-      <c r="I11" s="38"/>
-      <c r="J11" s="39"/>
-      <c r="K11" s="39" t="s">
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="29"/>
+      <c r="J11" s="30"/>
+      <c r="K11" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="L11" s="40" t="s">
+      <c r="L11" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="M11" s="38"/>
-      <c r="N11" s="39"/>
-      <c r="O11" s="41"/>
+      <c r="M11" s="29"/>
+      <c r="N11" s="30"/>
+      <c r="O11" s="32"/>
       <c r="T11" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:24" ht="145.19999999999999" x14ac:dyDescent="0.25">
-      <c r="A12" s="47">
+    <row r="12" spans="1:24" ht="118.8" x14ac:dyDescent="0.25">
+      <c r="A12" s="45">
         <v>2</v>
       </c>
-      <c r="B12" s="42">
-        <v>46174</v>
-      </c>
-      <c r="C12" s="43" t="s">
+      <c r="B12" s="54" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="D12" s="49" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
-      <c r="G12" s="43"/>
-      <c r="H12" s="43"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="43"/>
-      <c r="K12" s="43" t="s">
+      <c r="D12" s="52" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="34"/>
+      <c r="K12" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="L12" s="51" t="s">
+      <c r="L12" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="M12" s="42"/>
-      <c r="N12" s="43"/>
-      <c r="O12" s="44"/>
+      <c r="M12" s="33"/>
+      <c r="N12" s="34"/>
+      <c r="O12" s="35"/>
       <c r="T12" s="8" t="s">
         <v>23</v>
       </c>
@@ -1421,28 +1469,28 @@
       </c>
     </row>
     <row r="13" spans="1:24" ht="132" x14ac:dyDescent="0.25">
-      <c r="A13" s="47">
+      <c r="A13" s="45">
         <v>3</v>
       </c>
-      <c r="B13" s="42">
-        <v>46174</v>
-      </c>
-      <c r="C13" s="43" t="s">
+      <c r="B13" s="54" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="47" t="s">
         <v>67</v>
       </c>
-      <c r="D13" s="50" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="43"/>
-      <c r="H13" s="43"/>
-      <c r="I13" s="42"/>
-      <c r="J13" s="43"/>
-      <c r="K13" s="43" t="s">
+      <c r="D13" s="48" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="33"/>
+      <c r="J13" s="34"/>
+      <c r="K13" s="47" t="s">
         <v>22</v>
       </c>
-      <c r="L13" s="45" t="s">
+      <c r="L13" s="51" t="s">
         <v>70</v>
       </c>
       <c r="M13" s="10"/>
@@ -1461,21 +1509,31 @@
         <v>29</v>
       </c>
     </row>
-    <row r="14" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9">
+    <row r="14" spans="1:24" ht="257.39999999999998" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="45">
         <v>4</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="37"/>
+      <c r="B14" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="D14" s="48" t="s">
+        <v>77</v>
+      </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="10"/>
       <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
+      <c r="K14" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="L14" s="36" t="s">
+        <v>74</v>
+      </c>
       <c r="M14" s="10"/>
       <c r="N14" s="3"/>
       <c r="O14" s="12"/>
@@ -1492,21 +1550,31 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" ht="250.8" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>5</v>
       </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="11"/>
+      <c r="B15" s="54" t="s">
+        <v>72</v>
+      </c>
+      <c r="C15" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="52" t="s">
+        <v>78</v>
+      </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="10"/>
       <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
+      <c r="K15" s="47" t="s">
+        <v>22</v>
+      </c>
+      <c r="L15" s="51" t="s">
+        <v>79</v>
+      </c>
       <c r="M15" s="10"/>
       <c r="N15" s="3"/>
       <c r="O15" s="12"/>
@@ -1517,13 +1585,19 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" ht="215.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
         <v>6</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="11"/>
+      <c r="B16" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="52" t="s">
+        <v>80</v>
+      </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -1531,7 +1605,9 @@
       <c r="I16" s="10"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
+      <c r="L16" s="51" t="s">
+        <v>81</v>
+      </c>
       <c r="M16" s="10"/>
       <c r="N16" s="3"/>
       <c r="O16" s="12"/>
@@ -1542,13 +1618,19 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:24" ht="184.8" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>7</v>
       </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="11"/>
+      <c r="B17" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="47" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="52" t="s">
+        <v>82</v>
+      </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
@@ -1556,7 +1638,9 @@
       <c r="I17" s="10"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
+      <c r="L17" s="51" t="s">
+        <v>83</v>
+      </c>
       <c r="M17" s="10"/>
       <c r="N17" s="3"/>
       <c r="O17" s="12"/>
@@ -2856,7 +2940,7 @@
       </c>
     </row>
     <row r="10" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="34" t="s">
+      <c r="A10" s="42" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="25" t="s">
@@ -2864,19 +2948,19 @@
       </c>
     </row>
     <row r="11" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="35"/>
+      <c r="A11" s="43"/>
       <c r="B11" s="26" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="35"/>
+      <c r="A12" s="43"/>
       <c r="B12" s="26" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="36"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="26" t="s">
         <v>55</v>
       </c>

</xml_diff>